<commit_message>
Release v.03: start relocation middle band at 2000 sqm
</commit_message>
<xml_diff>
--- a/Negros/Negros_Pricing_Equal_Share.xlsx
+++ b/Negros/Negros_Pricing_Equal_Share.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Negros Pricing" sheetId="1" r:id="Red2c3e5a8d7849e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing Settings" sheetId="2" r:id="R54c22883f4184118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Negros Pricing" sheetId="1" r:id="Rc8eaa56480654808"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing Settings" sheetId="2" r:id="R5b31e6a9bcd6468d"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="Destinations">'Pricing Settings'!$G$7:$G$150</x:definedName>
@@ -557,7 +557,7 @@
         <x:color rgb="FF84909C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF0F2F4"/>
         </x:patternFill>
       </x:fill>
@@ -2151,7 +2151,7 @@
         <x:v>Middle band starts (sqm)</x:v>
       </x:c>
       <x:c r="C10" s="53" t="n">
-        <x:v>1000</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
         <x:v>Inclusive lower threshold.</x:v>

</xml_diff>